<commit_message>
Add raspberry pi-controlled relay circuit
</commit_message>
<xml_diff>
--- a/docs/anchor_DFMEA.xlsx
+++ b/docs/anchor_DFMEA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmatt\Documents\anchor\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F567E11-77FA-4AC8-8910-BED5E5D74DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEAA4534-711E-49CC-86BD-0B644BEB6096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{6E08087A-9028-4EA2-B63F-382C2D4CF040}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="AP_lookup_table" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2315" uniqueCount="1156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2315" uniqueCount="1159">
   <si>
     <t>Ref ID</t>
   </si>
@@ -3185,9 +3184,6 @@
     <t>Open circuit mains wire</t>
   </si>
   <si>
-    <t>Open circuit thermistor wire</t>
-  </si>
-  <si>
     <t>No power input to heater</t>
   </si>
   <si>
@@ -3495,6 +3491,18 @@
   </si>
   <si>
     <t>Metal Mount</t>
+  </si>
+  <si>
+    <t>Controller interprets temperature higher than actual</t>
+  </si>
+  <si>
+    <t>Open circuit PTC thermistor wire</t>
+  </si>
+  <si>
+    <t>Open circuit NTC thermistor wire</t>
+  </si>
+  <si>
+    <t>Software bug; Hardware failure / mosfet fused closed</t>
   </si>
 </sst>
 </file>
@@ -3623,6 +3631,12 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -3634,12 +3648,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4011,7 +4019,7 @@
     <col min="1" max="1" width="9.140625" style="2"/>
     <col min="2" max="2" width="18.140625" style="2" customWidth="1"/>
     <col min="3" max="3" width="18.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="26.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="30.28515625" style="1" customWidth="1"/>
     <col min="7" max="7" width="29.140625" style="1" customWidth="1"/>
@@ -4028,94 +4036,94 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>1098</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
+      <c r="A1" s="10" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
       <c r="P1" s="5"/>
     </row>
     <row r="2" spans="1:16" ht="93" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="12" t="s">
+      <c r="B2" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="8" t="s">
         <v>1031</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="8" t="s">
         <v>1032</v>
       </c>
-      <c r="H2" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" s="12" t="s">
+      <c r="H2" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="K2" s="12" t="s">
+      <c r="J2" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="8" t="s">
         <v>1050</v>
       </c>
-      <c r="L2" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="N2" s="12" t="s">
+      <c r="L2" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="N2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="O2" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="P2" s="13" t="s">
+      <c r="O2" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="P2" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
-        <v>1116</v>
-      </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="11"/>
+      <c r="A3" s="11" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="13"/>
     </row>
     <row r="4" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -4143,7 +4151,7 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="J4" s="4">
         <v>1</v>
@@ -4183,10 +4191,10 @@
         <v>1051</v>
       </c>
       <c r="E5" s="4" t="s">
+        <v>1052</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>1053</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>1054</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>1027</v>
@@ -4201,7 +4209,7 @@
         <v>2</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="L5" s="4">
         <v>2</v>
@@ -4211,7 +4219,7 @@
         <v>8</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="O5" s="4" t="s">
         <v>12</v>
@@ -4232,13 +4240,13 @@
         <v>5</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>1052</v>
+        <v>1157</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>1027</v>
@@ -4253,7 +4261,7 @@
         <v>2</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="L6" s="4">
         <v>2</v>
@@ -4263,10 +4271,10 @@
         <v>12</v>
       </c>
       <c r="N6" s="4" t="s">
+        <v>1056</v>
+      </c>
+      <c r="O6" s="4" t="s">
         <v>1057</v>
-      </c>
-      <c r="O6" s="4" t="s">
-        <v>1058</v>
       </c>
       <c r="P6" s="4" t="str">
         <f>VLOOKUP((H6&amp;J6&amp;L6),AP_lookup_table!D4:E1003,2,FALSE)</f>
@@ -4284,13 +4292,13 @@
         <v>5</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>1058</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>1059</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>1060</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>1061</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>1027</v>
@@ -4299,13 +4307,13 @@
         <v>7</v>
       </c>
       <c r="I7" s="4" t="s">
+        <v>1061</v>
+      </c>
+      <c r="J7" s="4">
+        <v>3</v>
+      </c>
+      <c r="K7" s="4" t="s">
         <v>1062</v>
-      </c>
-      <c r="J7" s="4">
-        <v>3</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>1063</v>
       </c>
       <c r="L7" s="4">
         <v>7</v>
@@ -4315,10 +4323,10 @@
         <v>147</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="P7" s="4" t="str">
         <f>VLOOKUP((H7&amp;J7&amp;L7),AP_lookup_table!D5:E1004,2,FALSE)</f>
@@ -4336,13 +4344,13 @@
         <v>5</v>
       </c>
       <c r="D8" s="4" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>1067</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>1068</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>1069</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>1027</v>
@@ -4351,13 +4359,13 @@
         <v>6</v>
       </c>
       <c r="I8" s="4" t="s">
+        <v>1069</v>
+      </c>
+      <c r="J8" s="4">
+        <v>2</v>
+      </c>
+      <c r="K8" s="4" t="s">
         <v>1070</v>
-      </c>
-      <c r="J8" s="4">
-        <v>2</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>1071</v>
       </c>
       <c r="L8" s="4">
         <v>3</v>
@@ -4367,10 +4375,10 @@
         <v>36</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="P8" s="4" t="str">
         <f>VLOOKUP((H8&amp;J8&amp;L8),AP_lookup_table!D6:E1005,2,FALSE)</f>
@@ -4391,25 +4399,25 @@
         <v>1047</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="H9" s="4">
         <v>8</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="J9" s="4">
         <v>1</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="L9" s="4">
         <v>5</v>
@@ -4419,10 +4427,10 @@
         <v>40</v>
       </c>
       <c r="N9" s="4" t="s">
+        <v>1076</v>
+      </c>
+      <c r="O9" s="4" t="s">
         <v>1077</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>1078</v>
       </c>
       <c r="P9" s="4" t="str">
         <f>VLOOKUP((H9&amp;J9&amp;L9),AP_lookup_table!D6:E1005,2,FALSE)</f>
@@ -4443,10 +4451,10 @@
         <v>1038</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>1027</v>
@@ -4461,7 +4469,7 @@
         <v>2</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="L10" s="4">
         <v>7</v>
@@ -4474,7 +4482,7 @@
         <v>12</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="P10" s="4" t="str">
         <f>VLOOKUP((H10&amp;J10&amp;L10),AP_lookup_table!D7:E1006,2,FALSE)</f>
@@ -4492,28 +4500,28 @@
         <v>1040</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="E11" s="4" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>1079</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="G11" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H11" s="4">
+        <v>10</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>1089</v>
+      </c>
+      <c r="J11" s="4">
+        <v>2</v>
+      </c>
+      <c r="K11" s="4" t="s">
         <v>1080</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="H11" s="4">
-        <v>10</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>1090</v>
-      </c>
-      <c r="J11" s="4">
-        <v>2</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>1081</v>
       </c>
       <c r="L11" s="4">
         <v>2</v>
@@ -4523,7 +4531,7 @@
         <v>40</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="O11" s="4" t="s">
         <v>12</v>
@@ -4544,13 +4552,13 @@
         <v>1040</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="E12" s="4" t="s">
+        <v>1090</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>1091</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>1092</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>1027</v>
@@ -4559,13 +4567,13 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J12" s="4">
         <v>1</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="L12" s="4">
         <v>1</v>
@@ -4575,7 +4583,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="O12" s="4" t="s">
         <v>12</v>
@@ -4587,7 +4595,7 @@
     </row>
     <row r="13" spans="1:16" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>1030</v>
@@ -4602,7 +4610,7 @@
         <v>1049</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>3</v>
@@ -4611,13 +4619,13 @@
         <v>10</v>
       </c>
       <c r="I13" s="4" t="s">
+        <v>1082</v>
+      </c>
+      <c r="J13" s="4">
+        <v>3</v>
+      </c>
+      <c r="K13" s="4" t="s">
         <v>1083</v>
-      </c>
-      <c r="J13" s="4">
-        <v>3</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>1084</v>
       </c>
       <c r="L13" s="4">
         <v>2</v>
@@ -4627,7 +4635,7 @@
         <v>60</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="O13" s="4" t="s">
         <v>12</v>
@@ -4648,28 +4656,28 @@
         <v>1041</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="E14" s="4" t="s">
+        <v>1100</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>1098</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>1099</v>
+      </c>
+      <c r="H14" s="4">
+        <v>6</v>
+      </c>
+      <c r="I14" s="4" t="s">
         <v>1101</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>1099</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>1100</v>
-      </c>
-      <c r="H14" s="4">
-        <v>6</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>1102</v>
-      </c>
       <c r="J14" s="4">
         <v>1</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="L14" s="4">
         <v>7</v>
@@ -4679,10 +4687,10 @@
         <v>42</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="O14" s="4" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="P14" s="4" t="str">
         <f>VLOOKUP((H14&amp;J14&amp;L14),AP_lookup_table!D11:E1010,2,FALSE)</f>
@@ -4690,34 +4698,34 @@
       </c>
     </row>
     <row r="15" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>1120</v>
-      </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="11"/>
+      <c r="A15" s="11" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="13"/>
     </row>
     <row r="16" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
@@ -4740,34 +4748,34 @@
       </c>
     </row>
     <row r="17" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
-        <v>1117</v>
-      </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
-      <c r="O17" s="10"/>
-      <c r="P17" s="11"/>
+      <c r="A17" s="11" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="13"/>
     </row>
     <row r="18" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>1114</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>1115</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>1028</v>
@@ -4785,7 +4793,7 @@
         <v>10</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="J18" s="4">
         <v>1</v>
@@ -4813,22 +4821,22 @@
     </row>
     <row r="19" spans="1:16" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>1114</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>1115</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>1051</v>
       </c>
       <c r="E19" s="4" t="s">
+        <v>1052</v>
+      </c>
+      <c r="F19" s="4" t="s">
         <v>1053</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>1054</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>1027</v>
@@ -4843,7 +4851,7 @@
         <v>2</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="L19" s="4">
         <v>2</v>
@@ -4853,7 +4861,7 @@
         <v>8</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="O19" s="4" t="s">
         <v>12</v>
@@ -4865,22 +4873,22 @@
     </row>
     <row r="20" spans="1:16" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>1114</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>1115</v>
-      </c>
       <c r="D20" s="4" t="s">
-        <v>1052</v>
+        <v>1156</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>1074</v>
+        <v>1155</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>1027</v>
@@ -4895,7 +4903,7 @@
         <v>2</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="L20" s="4">
         <v>2</v>
@@ -4905,10 +4913,10 @@
         <v>12</v>
       </c>
       <c r="N20" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="O20" s="4" t="s">
-        <v>1058</v>
+        <v>12</v>
       </c>
       <c r="P20" s="4" t="str">
         <f>VLOOKUP((H20&amp;J20&amp;L20),AP_lookup_table!D15:E1014,2,FALSE)</f>
@@ -4917,22 +4925,22 @@
     </row>
     <row r="21" spans="1:16" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>1114</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>1115</v>
-      </c>
       <c r="D21" s="4" t="s">
+        <v>1058</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>1059</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>1060</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>1061</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>1027</v>
@@ -4941,13 +4949,13 @@
         <v>7</v>
       </c>
       <c r="I21" s="4" t="s">
+        <v>1061</v>
+      </c>
+      <c r="J21" s="4">
+        <v>3</v>
+      </c>
+      <c r="K21" s="4" t="s">
         <v>1062</v>
-      </c>
-      <c r="J21" s="4">
-        <v>3</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>1063</v>
       </c>
       <c r="L21" s="4">
         <v>7</v>
@@ -4957,10 +4965,10 @@
         <v>147</v>
       </c>
       <c r="N21" s="4" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="P21" s="4" t="str">
         <f>VLOOKUP((H21&amp;J21&amp;L21),AP_lookup_table!D16:E1015,2,FALSE)</f>
@@ -4969,22 +4977,22 @@
     </row>
     <row r="22" spans="1:16" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>1114</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>1115</v>
-      </c>
       <c r="D22" s="4" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>1067</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="F22" s="4" t="s">
         <v>1068</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>1069</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>1027</v>
@@ -4993,13 +5001,13 @@
         <v>6</v>
       </c>
       <c r="I22" s="4" t="s">
+        <v>1069</v>
+      </c>
+      <c r="J22" s="4">
+        <v>2</v>
+      </c>
+      <c r="K22" s="4" t="s">
         <v>1070</v>
-      </c>
-      <c r="J22" s="4">
-        <v>2</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>1071</v>
       </c>
       <c r="L22" s="4">
         <v>3</v>
@@ -5009,10 +5017,10 @@
         <v>36</v>
       </c>
       <c r="N22" s="4" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="P22" s="4" t="str">
         <f>VLOOKUP((H22&amp;J22&amp;L22),AP_lookup_table!D17:E1016,2,FALSE)</f>
@@ -5021,19 +5029,19 @@
     </row>
     <row r="23" spans="1:16" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>1114</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>1115</v>
-      </c>
       <c r="D23" s="4" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>1145</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>1146</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>1027</v>
@@ -5045,13 +5053,13 @@
         <v>4</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="J23" s="4">
         <v>2</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="L23" s="4">
         <v>5</v>
@@ -5064,7 +5072,7 @@
         <v>12</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="P23" s="4" t="str">
         <f>VLOOKUP((H23&amp;J23&amp;L23),AP_lookup_table!D17:E1016,2,FALSE)</f>
@@ -5073,22 +5081,22 @@
     </row>
     <row r="24" spans="1:16" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>1038</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>1027</v>
@@ -5103,7 +5111,7 @@
         <v>2</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="L24" s="4">
         <v>7</v>
@@ -5116,7 +5124,7 @@
         <v>12</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="P24" s="4" t="str">
         <f>VLOOKUP((H24&amp;J24&amp;L24),AP_lookup_table!D18:E1017,2,FALSE)</f>
@@ -5125,37 +5133,37 @@
     </row>
     <row r="25" spans="1:16" ht="66.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>1040</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="E25" s="4" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F25" s="4" t="s">
         <v>1079</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="G25" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H25" s="4">
+        <v>10</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>1089</v>
+      </c>
+      <c r="J25" s="4">
+        <v>2</v>
+      </c>
+      <c r="K25" s="4" t="s">
         <v>1080</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="H25" s="4">
-        <v>10</v>
-      </c>
-      <c r="I25" s="4" t="s">
-        <v>1090</v>
-      </c>
-      <c r="J25" s="4">
-        <v>2</v>
-      </c>
-      <c r="K25" s="4" t="s">
-        <v>1081</v>
       </c>
       <c r="L25" s="4">
         <v>2</v>
@@ -5165,7 +5173,7 @@
         <v>40</v>
       </c>
       <c r="N25" s="4" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="O25" s="4" t="s">
         <v>12</v>
@@ -5177,22 +5185,22 @@
     </row>
     <row r="26" spans="1:16" ht="66.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>1040</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="E26" s="4" t="s">
+        <v>1090</v>
+      </c>
+      <c r="F26" s="4" t="s">
         <v>1091</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>1092</v>
       </c>
       <c r="G26" s="4" t="s">
         <v>1027</v>
@@ -5201,13 +5209,13 @@
         <v>1</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J26" s="4">
         <v>1</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="L26" s="4">
         <v>1</v>
@@ -5217,7 +5225,7 @@
         <v>1</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="O26" s="4" t="s">
         <v>12</v>
@@ -5229,10 +5237,10 @@
     </row>
     <row r="27" spans="1:16" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>1040</v>
@@ -5244,7 +5252,7 @@
         <v>1049</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>3</v>
@@ -5253,13 +5261,13 @@
         <v>10</v>
       </c>
       <c r="I27" s="4" t="s">
+        <v>1082</v>
+      </c>
+      <c r="J27" s="4">
+        <v>3</v>
+      </c>
+      <c r="K27" s="4" t="s">
         <v>1083</v>
-      </c>
-      <c r="J27" s="4">
-        <v>3</v>
-      </c>
-      <c r="K27" s="4" t="s">
-        <v>1084</v>
       </c>
       <c r="L27" s="4">
         <v>2</v>
@@ -5269,7 +5277,7 @@
         <v>60</v>
       </c>
       <c r="N27" s="4" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="O27" s="4" t="s">
         <v>12</v>
@@ -5281,37 +5289,37 @@
     </row>
     <row r="28" spans="1:16" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>1041</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="E28" s="4" t="s">
+        <v>1100</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>1098</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>1099</v>
+      </c>
+      <c r="H28" s="4">
+        <v>6</v>
+      </c>
+      <c r="I28" s="4" t="s">
         <v>1101</v>
       </c>
-      <c r="F28" s="4" t="s">
-        <v>1099</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>1100</v>
-      </c>
-      <c r="H28" s="4">
-        <v>6</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>1102</v>
-      </c>
       <c r="J28" s="4">
         <v>1</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="L28" s="4">
         <v>7</v>
@@ -5321,10 +5329,10 @@
         <v>42</v>
       </c>
       <c r="N28" s="4" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="O28" s="4" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="P28" s="4" t="str">
         <f>VLOOKUP((H28&amp;J28&amp;L28),AP_lookup_table!D22:E1021,2,FALSE)</f>
@@ -5333,37 +5341,37 @@
     </row>
     <row r="29" spans="1:16" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>1133</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>1114</v>
-      </c>
-      <c r="C29" s="4" t="s">
+      <c r="D29" s="4" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>1138</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>1139</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>1140</v>
+      </c>
+      <c r="H29" s="4">
+        <v>5</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>1136</v>
+      </c>
+      <c r="J29" s="4">
+        <v>3</v>
+      </c>
+      <c r="K29" s="4" t="s">
         <v>1134</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>1136</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>1139</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>1140</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>1141</v>
-      </c>
-      <c r="H29" s="4">
-        <v>5</v>
-      </c>
-      <c r="I29" s="4" t="s">
-        <v>1137</v>
-      </c>
-      <c r="J29" s="4">
-        <v>3</v>
-      </c>
-      <c r="K29" s="4" t="s">
-        <v>1135</v>
       </c>
       <c r="L29" s="4">
         <v>2</v>
@@ -5373,7 +5381,7 @@
         <v>30</v>
       </c>
       <c r="N29" s="4" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="O29" s="4" t="s">
         <v>12</v>
@@ -5384,43 +5392,43 @@
       </c>
     </row>
     <row r="30" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="9" t="s">
-        <v>1118</v>
-      </c>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="10"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="10"/>
-      <c r="P30" s="11"/>
+      <c r="A30" s="11" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="12"/>
+      <c r="M30" s="12"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="12"/>
+      <c r="P30" s="13"/>
     </row>
     <row r="31" spans="1:16" ht="111" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>1104</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="C31" s="4" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>1105</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>1106</v>
-      </c>
       <c r="E31" s="4" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>3</v>
@@ -5429,13 +5437,13 @@
         <v>10</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>1109</v>
+        <v>1158</v>
       </c>
       <c r="J31" s="4">
         <v>2</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="L31" s="4">
         <v>1</v>
@@ -5457,22 +5465,22 @@
     </row>
     <row r="32" spans="1:16" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>1027</v>
@@ -5481,13 +5489,13 @@
         <v>1</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="J32" s="4">
         <v>1</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="L32" s="4">
         <v>3</v>
@@ -5509,37 +5517,37 @@
     </row>
     <row r="33" spans="1:16" ht="116.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>1111</v>
       </c>
-      <c r="B33" s="4" t="s">
-        <v>1105</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>1112</v>
-      </c>
       <c r="D33" s="4" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="E33" s="4" t="s">
+        <v>1147</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>1151</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H33" s="4">
+        <v>10</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>1150</v>
+      </c>
+      <c r="J33" s="4">
+        <v>2</v>
+      </c>
+      <c r="K33" s="4" t="s">
         <v>1148</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>1152</v>
-      </c>
-      <c r="G33" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="H33" s="4">
-        <v>10</v>
-      </c>
-      <c r="I33" s="4" t="s">
-        <v>1151</v>
-      </c>
-      <c r="J33" s="4">
-        <v>2</v>
-      </c>
-      <c r="K33" s="4" t="s">
-        <v>1149</v>
       </c>
       <c r="L33" s="4">
         <v>1</v>
@@ -6271,6 +6279,18 @@
   </mergeCells>
   <conditionalFormatting sqref="H4:H16 J4:J16 L4:L16 L18:L29 J18:J29 H18:H29 L31:L125 H31:H125 J31:J125">
     <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="num" val="1"/>
+        <cfvo type="num" val="5"/>
+        <cfvo type="num" val="10"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L16 J16 H16">
+    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="num" val="1"/>
         <cfvo type="num" val="5"/>
@@ -6293,29 +6313,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P4:P16 P18:P29 P31:P125">
-    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
-      <formula>"H"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="8" operator="equal">
-      <formula>"M"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="9" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J16 L16 H16">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="num" val="1"/>
-        <cfvo type="num" val="5"/>
-        <cfvo type="num" val="10"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="M16">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -6328,14 +6325,25 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P16">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+  <conditionalFormatting sqref="P4:P16">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"H"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>"M"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P18:P29 P31:P125">
+    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
+      <formula>"H"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
+      <formula>"M"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
       <formula>"L"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>